<commit_message>
Post Upload validation via UI Search
</commit_message>
<xml_diff>
--- a/ResourcesPK/configPK.xlsx
+++ b/ResourcesPK/configPK.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="182">
   <si>
     <t>screenName</t>
   </si>
@@ -518,13 +518,67 @@
   </si>
   <si>
     <t>Selling_Category_Bulk_Upload.xlsx</t>
+  </si>
+  <si>
+    <t>validateMode</t>
+  </si>
+  <si>
+    <t>validateScreenId</t>
+  </si>
+  <si>
+    <t>DYL_202044</t>
+  </si>
+  <si>
+    <t>menuSearch</t>
+  </si>
+  <si>
+    <t>UI_Search</t>
+  </si>
+  <si>
+    <t>dsr profile hq</t>
+  </si>
+  <si>
+    <t>validateGeneratedCol</t>
+  </si>
+  <si>
+    <t>columnId</t>
+  </si>
+  <si>
+    <t>DYL_BG1013</t>
+  </si>
+  <si>
+    <t>Outlet profile HQ</t>
+  </si>
+  <si>
+    <t>rowfilter_TXT__EPP1DESC</t>
+  </si>
+  <si>
+    <t>User profile</t>
+  </si>
+  <si>
+    <t>0201</t>
+  </si>
+  <si>
+    <t>rowfilter_code</t>
+  </si>
+  <si>
+    <t>Vehicle Profile</t>
+  </si>
+  <si>
+    <t>DYL_1032</t>
+  </si>
+  <si>
+    <t>rowfilter_Description</t>
+  </si>
+  <si>
+    <t>rowfilter_TXT__EPP2DESC</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -536,6 +590,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -567,7 +627,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -614,11 +674,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -662,6 +731,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -942,7 +1023,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr defaultColWidth="31.54296875" defaultRowHeight="15.65" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.7265625" customWidth="1"/>
@@ -953,7 +1034,7 @@
     <col min="6" max="6" width="10.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="8" t="s">
         <v>106</v>
       </c>
@@ -972,8 +1053,23 @@
       <c r="F1" s="9" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" s="6" customFormat="1" ht="23.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G1" s="25" t="s">
+        <v>164</v>
+      </c>
+      <c r="H1" s="25" t="s">
+        <v>167</v>
+      </c>
+      <c r="I1" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="J1" s="25" t="s">
+        <v>170</v>
+      </c>
+      <c r="K1" s="25" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" s="6" customFormat="1" ht="23.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="10" t="s">
         <v>107</v>
       </c>
@@ -992,8 +1088,23 @@
       <c r="F2" s="11" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" s="23" customFormat="1" ht="32.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G2" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" s="23" customFormat="1" ht="32.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="21" t="s">
         <v>108</v>
       </c>
@@ -1013,7 +1124,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="4" spans="1:6" s="6" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" s="6" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="10" t="s">
         <v>109</v>
       </c>
@@ -1033,7 +1144,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="5" spans="1:6" s="6" customFormat="1" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" s="6" customFormat="1" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="10" t="s">
         <v>111</v>
       </c>
@@ -1050,10 +1161,25 @@
         <v>60</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+        <v>78</v>
+      </c>
+      <c r="G5" s="19" t="s">
+        <v>168</v>
+      </c>
+      <c r="H5" s="19" t="s">
+        <v>173</v>
+      </c>
+      <c r="I5" s="26" t="s">
+        <v>172</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="10" t="s">
         <v>112</v>
       </c>
@@ -1070,10 +1196,13 @@
         <v>61</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" s="6" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+        <v>133</v>
+      </c>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19"/>
+      <c r="I6" s="26"/>
+    </row>
+    <row r="7" spans="1:11" s="6" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
         <v>113</v>
       </c>
@@ -1093,7 +1222,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="8" spans="1:6" s="6" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" s="6" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="10" t="s">
         <v>114</v>
       </c>
@@ -1113,7 +1242,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="9" spans="1:6" s="6" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" s="6" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
         <v>115</v>
       </c>
@@ -1133,7 +1262,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="10" spans="1:6" s="6" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" s="6" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="10" t="s">
         <v>116</v>
       </c>
@@ -1153,7 +1282,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
         <v>117</v>
       </c>
@@ -1173,7 +1302,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="10" t="s">
         <v>118</v>
       </c>
@@ -1193,7 +1322,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="13" t="s">
         <v>120</v>
       </c>
@@ -1213,7 +1342,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="14" spans="1:6" s="16" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" s="16" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="10" t="s">
         <v>122</v>
       </c>
@@ -1233,7 +1362,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="17" t="s">
         <v>126</v>
       </c>
@@ -1253,7 +1382,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="16" spans="1:6" s="6" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" s="6" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="10" t="s">
         <v>110</v>
       </c>
@@ -1271,7 +1400,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="13" t="s">
         <v>134</v>
       </c>
@@ -1282,16 +1411,31 @@
         <v>92</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E17" s="15" t="s">
         <v>135</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" s="16" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+        <v>78</v>
+      </c>
+      <c r="G17" s="19" t="s">
+        <v>168</v>
+      </c>
+      <c r="H17" s="19" t="s">
+        <v>178</v>
+      </c>
+      <c r="I17" s="28" t="s">
+        <v>179</v>
+      </c>
+      <c r="J17" s="26" t="s">
+        <v>136</v>
+      </c>
+      <c r="K17" s="27" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" s="16" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="20" t="s">
         <v>140</v>
       </c>
@@ -1311,7 +1455,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="19" spans="1:6" s="16" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" s="16" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="20" t="s">
         <v>149</v>
       </c>
@@ -1331,7 +1475,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="20" t="s">
         <v>152</v>
       </c>
@@ -1348,10 +1492,25 @@
         <v>159</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+        <v>78</v>
+      </c>
+      <c r="G20" s="19" t="s">
+        <v>168</v>
+      </c>
+      <c r="H20" s="19" t="s">
+        <v>175</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="J20" s="26" t="s">
+        <v>155</v>
+      </c>
+      <c r="K20" s="26" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="24" t="s">
         <v>160</v>
       </c>
@@ -1483,7 +1642,7 @@
       </c>
       <c r="D7" s="4" t="str">
         <f ca="1" xml:space="preserve"> TEXT(TODAY() - 4, "yyyy-mm-dd")</f>
-        <v>2026-05-07</v>
+        <v>2026-05-09</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1498,7 +1657,7 @@
       </c>
       <c r="D8" s="5" t="str">
         <f ca="1">TEXT(TODAY()+2, "yyyy-mm-dd")</f>
-        <v>2026-05-13</v>
+        <v>2026-05-15</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>